<commit_message>
scan: seg6 2026-07-21 17:30 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-21.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-21.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3601,21 +3601,21 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6556</v>
+        <v>6831</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>邁科</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>423.8657062368541</v>
+        <v>424.9984064240117</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>65.5</v>
+        <v>600</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>28.99645603074997</v>
+        <v>37.85251831622244</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>30.26765623569774</v>
+        <v>26.95538513740867</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.41625078162791</v>
+        <v>0.3620515204491001</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.7212508598952969</v>
+        <v>-33.59888447232714</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6788</v>
+        <v>6556</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>423.4359649170433</v>
+        <v>423.8657062368541</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>354</v>
+        <v>65.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>35.42530278923827</v>
+        <v>28.99645603074997</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>22.17076457916664</v>
+        <v>30.26765623569774</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.2896542742394305</v>
+        <v>1.41625078162791</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-8.230627972110856</v>
+        <v>-0.7212508598952969</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6807</v>
+        <v>6788</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>416.8079004546015</v>
+        <v>423.4359649170433</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>33.95</v>
+        <v>354</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>55.12640093430798</v>
+        <v>35.42530278923827</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>10.87786625089214</v>
+        <v>22.17076457916664</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.2352315144496005</v>
+        <v>0.2896542742394305</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.1023627871298943</v>
+        <v>-8.230627972110856</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6577</v>
+        <v>6807</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>勁豐</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>411.5022347994853</v>
+        <v>416.8079004546015</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>76.5</v>
+        <v>33.95</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>48.28058788515763</v>
+        <v>55.12640093430798</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>18.4338393772652</v>
+        <v>10.87786625089214</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.3911171324270953</v>
+        <v>0.2352315144496005</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0514361514203826</v>
+        <v>0.1023627871298943</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6683</v>
+        <v>6577</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>雍智科技</t>
+          <t>勁豐</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>410.9492062215872</v>
+        <v>411.5022347994853</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>1170</v>
+        <v>76.5</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,49 +3838,49 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>31.90523531838022</v>
+        <v>48.28058788515763</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>18.60224394656252</v>
+        <v>18.4338393772652</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.011494319055256</v>
+        <v>0.3911171324270953</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M64" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-64.8597621703519</v>
+        <v>0.0514361514203826</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6641</v>
+        <v>6683</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>雍智科技</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>406.8796954157538</v>
+        <v>410.9492062215872</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>18</v>
+        <v>1170</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,49 +3891,49 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.55846354164191</v>
+        <v>31.90523531838022</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>15.68337735579495</v>
+        <v>18.60224394656252</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.4984131778668877</v>
+        <v>1.011494319055256</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M65" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.061849264017184</v>
+        <v>-64.8597621703519</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6716</v>
+        <v>6641</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>應廣</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>403.2825004304004</v>
+        <v>406.8796954157538</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>38.39130180262156</v>
+        <v>45.55846354164191</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>19.53481185785543</v>
+        <v>15.68337735579495</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.2722399287107146</v>
+        <v>0.4984131778668877</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-1.900180870928118</v>
+        <v>-0.061849264017184</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6588</v>
+        <v>6716</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>應廣</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>402.0560678062517</v>
+        <v>403.2825004304004</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>69.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>26.80607491988586</v>
+        <v>38.39130180262156</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>28.90642126046385</v>
+        <v>19.53481185785543</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.4336938881615549</v>
+        <v>0.2722399287107146</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.3464745984586077</v>
+        <v>-1.900180870928118</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6532</v>
+        <v>6588</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>401.7470053023894</v>
+        <v>402.0560678062517</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>69.59999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>29.37068839980262</v>
+        <v>26.80607491988586</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>27.88942803648954</v>
+        <v>28.90642126046385</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.2464462822837645</v>
+        <v>0.4336938881615549</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-1.431550517369997</v>
+        <v>-0.3464745984586077</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6643</v>
+        <v>6532</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>396.8334219806272</v>
+        <v>401.7470053023894</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>419.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>38.63621356183378</v>
+        <v>29.37068839980262</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>22.76976789820991</v>
+        <v>27.88942803648954</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1.286484397627313</v>
+        <v>0.2464462822837645</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-2.469736369657205</v>
+        <v>-1.431550517369997</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6504</v>
+        <v>6643</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>南六</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>396.71598081606</v>
+        <v>396.8334219806272</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>36.4</v>
+        <v>419.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>50.82409037729572</v>
+        <v>38.63621356183378</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>12.1908549890605</v>
+        <v>22.76976789820991</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.7910643082744567</v>
+        <v>1.286484397627313</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.1080913383644848</v>
+        <v>-2.469736369657205</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6803</v>
+        <v>6504</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>南六</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>385.3711079848118</v>
+        <v>396.71598081606</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>271.5</v>
+        <v>36.4</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>34.87077048097069</v>
+        <v>50.82409037729572</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>46.78125379395011</v>
+        <v>12.1908549890605</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.4140140579481616</v>
+        <v>0.7910643082744567</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.8963376929934621</v>
+        <v>0.1080913383644848</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6642</v>
+        <v>6803</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>富致</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>382.2060193045441</v>
+        <v>385.3711079848118</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>74.40000000000001</v>
+        <v>271.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>40.88234220771578</v>
+        <v>34.87077048097069</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.9724865586012</v>
+        <v>46.78125379395011</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.2271409856917009</v>
+        <v>0.4140140579481616</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-1.056823077188846</v>
+        <v>-0.8963376929934621</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6727</v>
+        <v>6642</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>亞泰金屬</t>
+          <t>富致</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>379.870443554066</v>
+        <v>382.2060193045441</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>332.5</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>34.86415868024959</v>
+        <v>40.88234220771578</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.9389935407248</v>
+        <v>22.9724865586012</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.5816082988866277</v>
+        <v>0.2271409856917009</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-13.53669422381942</v>
+        <v>-1.056823077188846</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6550</v>
+        <v>6727</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>北極星藥業-KY</t>
+          <t>亞泰金屬</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>378.7024064110562</v>
+        <v>379.870443554066</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>12.4</v>
+        <v>332.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>40.05177007078344</v>
+        <v>34.86415868024959</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>20.68512534836017</v>
+        <v>15.9389935407248</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.5240446479290128</v>
+        <v>0.5816082988866277</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.0075741551895148</v>
+        <v>-13.53669422381942</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6763</v>
+        <v>6550</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>北極星藥業-KY</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>370.2592313870658</v>
+        <v>378.7024064110562</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>42.55</v>
+        <v>12.4</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,16 +4421,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>35.64893980967128</v>
+        <v>40.05177007078344</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>24.42530370767916</v>
+        <v>20.68512534836017</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.3224486854768</v>
+        <v>0.5240446479290128</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.4265845855023487</v>
+        <v>-0.0075741551895148</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6530</v>
+        <v>6763</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>362.486669992194</v>
+        <v>370.2592313870658</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>69.8</v>
+        <v>42.55</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>26.97326350715653</v>
+        <v>35.64893980967128</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>30.88349403150102</v>
+        <v>24.42530370767916</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.4436135109391801</v>
+        <v>0.3224486854768</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.9842706462132388</v>
+        <v>-0.4265845855023487</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6679</v>
+        <v>6530</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>鈺太</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>359.0737410045408</v>
+        <v>362.486669992194</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>226</v>
+        <v>69.8</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>33.39407226334804</v>
+        <v>26.97326350715653</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>30.44386775006022</v>
+        <v>30.88349403150102</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.7644431746325844</v>
+        <v>0.4436135109391801</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-2.777727142458861</v>
+        <v>-0.9842706462132388</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4555,21 +4555,21 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6541</v>
+        <v>6679</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>鈺太</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>354.8766087358665</v>
+        <v>359.0737410045408</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>40.4</v>
+        <v>226</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>50.39820638670356</v>
+        <v>33.39407226334804</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>13.08170810185162</v>
+        <v>30.44386775006022</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.5860817169954384</v>
+        <v>0.7644431746325844</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.1533594480234193</v>
+        <v>-2.777727142458861</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6761</v>
+        <v>6541</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>349.8639486136669</v>
+        <v>354.8766087358665</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>156</v>
+        <v>40.4</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>34.27820243704154</v>
+        <v>50.39820638670356</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>20.05032917933261</v>
+        <v>13.08170810185162</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.4361879505926375</v>
+        <v>0.5860817169954384</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-3.423024377479662</v>
+        <v>-0.1533594480234193</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6782</v>
+        <v>6761</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>視陽</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>349.0318901902074</v>
+        <v>349.8639486136669</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>194.5</v>
+        <v>156</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>44.73037225611677</v>
+        <v>34.27820243704154</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.8683908397432</v>
+        <v>20.05032917933261</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>1.061360774142251</v>
+        <v>0.4361879505926375</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-1.062063943772525</v>
+        <v>-3.423024377479662</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6515</v>
+        <v>6782</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>視陽</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>348.3428505511702</v>
+        <v>349.0318901902074</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>6655</v>
+        <v>194.5</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>37.80137149894402</v>
+        <v>44.73037225611677</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>22.99345905570239</v>
+        <v>14.8683908397432</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>1.271380595490554</v>
+        <v>1.061360774142251</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-209.4269459201975</v>
+        <v>-1.062063943772525</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6498</v>
+        <v>6515</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>348.2386530011707</v>
+        <v>348.3428505511702</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>80.3</v>
+        <v>6655</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>29.51390079900932</v>
+        <v>37.80137149894402</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.94256350217949</v>
+        <v>22.99345905570239</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.5839952022855086</v>
+        <v>1.271380595490554</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-1.155772168691913</v>
+        <v>-209.4269459201975</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6770</v>
+        <v>6498</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>348.0960050229002</v>
+        <v>348.2386530011707</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>65.09999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>41.5930660817591</v>
+        <v>29.51390079900932</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>14.50310172010831</v>
+        <v>27.94256350217949</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.5197728290022108</v>
+        <v>0.5839952022855086</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-1.230256387263857</v>
+        <v>-1.155772168691913</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6768</v>
+        <v>6770</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>347.6234244969842</v>
+        <v>348.0960050229002</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>69.5</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>26.03997595932768</v>
+        <v>41.5930660817591</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>34.72102109364683</v>
+        <v>14.50310172010831</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1.12005424972941</v>
+        <v>0.5197728290022108</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0082915031616153</v>
+        <v>-1.230256387263857</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6510</v>
+        <v>6768</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>345.9317851533083</v>
+        <v>347.6234244969842</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>2645</v>
+        <v>69.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,49 +4951,49 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>36.55746253893226</v>
+        <v>26.03997595932768</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>28.73216519055497</v>
+        <v>34.72102109364683</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5658044009280173</v>
+        <v>1.12005424972941</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M85" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-35.55023145449491</v>
+        <v>-0.0082915031616153</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6821</v>
+        <v>6510</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>聯寶</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>345.5675431357321</v>
+        <v>345.9317851533083</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>43.6</v>
+        <v>2645</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,25 +5004,25 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>24.87041808831165</v>
+        <v>36.55746253893226</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>24.06611086980465</v>
+        <v>28.73216519055497</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.1699145537406587</v>
+        <v>0.5658044009280173</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M86" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-1.452088320715968</v>
+        <v>-35.55023145449491</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5032,21 +5032,21 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6754</v>
+        <v>6821</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>聯寶</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>345.4582780492537</v>
+        <v>345.5675431357321</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>42.15</v>
+        <v>43.6</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>40.7354461353418</v>
+        <v>24.87041808831165</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>13.45796734741536</v>
+        <v>24.06611086980465</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.6966227931904161</v>
+        <v>0.1699145537406587</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.0832193686756891</v>
+        <v>-1.452088320715968</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6706</v>
+        <v>6754</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>341.6697855786101</v>
+        <v>345.4582780492537</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>109.5</v>
+        <v>42.15</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>28.11280463106641</v>
+        <v>40.7354461353418</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>27.37460546190276</v>
+        <v>13.45796734741536</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.5923693021199806</v>
+        <v>0.6966227931904161</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-3.040458260957681</v>
+        <v>-0.0832193686756891</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6741</v>
+        <v>6706</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>340.384901843666</v>
+        <v>341.6697855786101</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>55.7</v>
+        <v>109.5</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>29.6035497419028</v>
+        <v>28.11280463106641</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>24.05610387740028</v>
+        <v>27.37460546190276</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>2.4384901843666</v>
+        <v>0.5923693021199806</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.3982184168858345</v>
+        <v>-3.040458260957681</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6799</v>
+        <v>6741</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>來頡</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>339.1705082565118</v>
+        <v>340.384901843666</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>84.2</v>
+        <v>55.7</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>38.38017394729031</v>
+        <v>29.6035497419028</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>22.47944420971817</v>
+        <v>24.05610387740028</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.2298645334558501</v>
+        <v>2.4384901843666</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-2.279124931987616</v>
+        <v>-0.3982184168858345</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6494</v>
+        <v>6799</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>九齊</t>
+          <t>來頡</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>333.598697378827</v>
+        <v>339.1705082565118</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>51.3</v>
+        <v>84.2</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>32.73046340624782</v>
+        <v>38.38017394729031</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>28.99549582969402</v>
+        <v>22.47944420971817</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.2725110198726092</v>
+        <v>0.2298645334558501</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-2.10763680817153</v>
+        <v>-2.279124931987616</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6667</v>
+        <v>6494</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>九齊</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>333.4025503488107</v>
+        <v>333.598697378827</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>241</v>
+        <v>51.3</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,16 +5322,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>35.37296221741435</v>
+        <v>32.73046340624782</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>16.86296986624651</v>
+        <v>28.99549582969402</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.2566204569731286</v>
+        <v>0.2725110198726092</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.563020659585904</v>
+        <v>-2.10763680817153</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6823</v>
+        <v>6667</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>濾能</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>332.7511727008838</v>
+        <v>333.4025503488107</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>61.3</v>
+        <v>241</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,16 +5375,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.22445199398146</v>
+        <v>35.37296221741435</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>15.71886608759834</v>
+        <v>16.86296986624651</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1.008527850135887</v>
+        <v>0.2566204569731286</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.4419458438973096</v>
+        <v>-2.563020659585904</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6698</v>
+        <v>6823</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>濾能</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>329.0812427752085</v>
+        <v>332.7511727008838</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>34.5</v>
+        <v>61.3</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>34.35470148409861</v>
+        <v>35.22445199398146</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>21.82768085541173</v>
+        <v>15.71886608759834</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.1820334187830753</v>
+        <v>1.008527850135887</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-1.044994624319222</v>
+        <v>-0.4419458438973096</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6725</v>
+        <v>6698</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>矽科宏晟</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>327.0531676681106</v>
+        <v>329.0812427752085</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>301</v>
+        <v>34.5</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.01941748042877</v>
+        <v>34.35470148409861</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.99863491105409</v>
+        <v>21.82768085541173</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.2078119067902938</v>
+        <v>0.1820334187830753</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-3.503879884285017</v>
+        <v>-1.044994624319222</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6735</v>
+        <v>6725</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>美達科技</t>
+          <t>矽科宏晟</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>322.1283171803583</v>
+        <v>327.0531676681106</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>66.59999999999999</v>
+        <v>301</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>21.94099963245938</v>
+        <v>44.01941748042877</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>23.2844035465303</v>
+        <v>15.99863491105409</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.482384711414239</v>
+        <v>0.2078119067902938</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-1.254643375406501</v>
+        <v>-3.503879884285017</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6796</v>
+        <v>6735</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>晉弘</t>
+          <t>美達科技</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>320.5640632746843</v>
+        <v>322.1283171803583</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>57.9</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>45.59826965444908</v>
+        <v>21.94099963245938</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>17.08564057553528</v>
+        <v>23.2844035465303</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.5287900689479289</v>
+        <v>0.482384711414239</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.1604558156868044</v>
+        <v>-1.254643375406501</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6560</v>
+        <v>6796</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>晉弘</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>319.439950225518</v>
+        <v>320.5640632746843</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>34</v>
+        <v>57.9</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>35.59245173280742</v>
+        <v>45.59826965444908</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>26.24215898666021</v>
+        <v>17.08564057553528</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.6916524796454414</v>
+        <v>0.5287900689479289</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.5822032295889031</v>
+        <v>0.1604558156868044</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6605</v>
+        <v>6560</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>318.6761640363342</v>
+        <v>319.439950225518</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>44.50624077783105</v>
+        <v>35.59245173280742</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.43801017560708</v>
+        <v>26.24215898666021</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.5080011550765238</v>
+        <v>0.6916524796454414</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.3589889297372031</v>
+        <v>-0.5822032295889031</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6742</v>
+        <v>6605</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>澤米</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>318.5809490122728</v>
+        <v>318.6761640363342</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>44.9</v>
+        <v>131</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>28.65558534224053</v>
+        <v>44.50624077783105</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>23.00948872606743</v>
+        <v>16.43801017560708</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.231461840980901</v>
+        <v>0.5080011550765238</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-2.384213471751985</v>
+        <v>-0.3589889297372031</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6794</v>
+        <v>6742</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>澤米</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>311.7969393121355</v>
+        <v>318.5809490122728</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>77.5</v>
+        <v>44.9</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.96796759205556</v>
+        <v>28.65558534224053</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>15.3326954786821</v>
+        <v>23.00948872606743</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.4663113213299086</v>
+        <v>0.231461840980901</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.3854888210935939</v>
+        <v>-2.384213471751985</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6689</v>
+        <v>6794</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>305.9930893135564</v>
+        <v>311.7969393121355</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>62.1</v>
+        <v>77.5</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.88373781461073</v>
+        <v>42.96796759205556</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>19.74586533855715</v>
+        <v>15.3326954786821</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.4064735811237634</v>
+        <v>0.4663113213299086</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.1080941637103485</v>
+        <v>-0.3854888210935939</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6581</v>
+        <v>6689</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>297.3050165789065</v>
+        <v>305.9930893135564</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>107</v>
+        <v>62.1</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>46.3717540659685</v>
+        <v>41.88373781461073</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>9.421248994043609</v>
+        <v>19.74586533855715</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>1.899794256570749</v>
+        <v>0.4064735811237634</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.07867441422863911</v>
+        <v>-0.1080941637103485</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6584</v>
+        <v>6581</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>295.4383182791996</v>
+        <v>297.3050165789065</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>541</v>
+        <v>107</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>33.44180901794688</v>
+        <v>46.3717540659685</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>16.85164301449299</v>
+        <v>9.421248994043609</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.3387083642598109</v>
+        <v>1.899794256570749</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-17.41468016369804</v>
+        <v>0.07867441422863911</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6781</v>
+        <v>6584</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>294.6060468779157</v>
+        <v>295.4383182791996</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>969</v>
+        <v>541</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>35.51576458158844</v>
+        <v>33.44180901794688</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.48966108486044</v>
+        <v>16.85164301449299</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.3614266888017936</v>
+        <v>0.3387083642598109</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-25.08842026830434</v>
+        <v>-17.41468016369804</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6589</v>
+        <v>6781</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>台康生技</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>294.127703998691</v>
+        <v>294.6060468779157</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>45.5</v>
+        <v>969</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>45.43278012067141</v>
+        <v>35.51576458158844</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>20.01362868060879</v>
+        <v>18.48966108486044</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.2794278286585127</v>
+        <v>0.3614266888017936</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.5699217018416459</v>
+        <v>-25.08842026830434</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6792</v>
+        <v>6589</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>台康生技</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>287.0724820749576</v>
+        <v>294.127703998691</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>54</v>
+        <v>45.5</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>32.74030460383599</v>
+        <v>45.43278012067141</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>20.81084491014651</v>
+        <v>20.01362868060879</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.5578760292888586</v>
+        <v>0.2794278286585127</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-1.088935891650083</v>
+        <v>-0.5699217018416459</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6655</v>
+        <v>6792</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>科定</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>285.9642288871706</v>
+        <v>287.0724820749576</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>117.5</v>
+        <v>54</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>48.81668572077849</v>
+        <v>32.74030460383599</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>6.38953664618426</v>
+        <v>20.81084491014651</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.2397048004680557</v>
+        <v>0.5578760292888586</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.3938931559076561</v>
+        <v>-1.088935891650083</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6720</v>
+        <v>6655</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>科定</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>268.99741920835</v>
+        <v>285.9642288871706</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>138</v>
+        <v>117.5</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>41.96945217471609</v>
+        <v>48.81668572077849</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>21.16627461687613</v>
+        <v>6.38953664618426</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.9766484197992292</v>
+        <v>0.2397048004680557</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.1189319696934552</v>
+        <v>0.3938931559076561</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6526</v>
+        <v>6720</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>263.4628012243699</v>
+        <v>268.99741920835</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>584</v>
+        <v>138</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>39.98426959269487</v>
+        <v>41.96945217471609</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>15.24099070834628</v>
+        <v>21.16627461687613</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.4249356230263151</v>
+        <v>0.9766484197992292</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-12.88473165907399</v>
+        <v>0.1189319696934552</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6756</v>
+        <v>6526</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>262.9967487218146</v>
+        <v>263.4628012243699</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>94</v>
+        <v>584</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>45.33000307534098</v>
+        <v>39.98426959269487</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.79812087559853</v>
+        <v>15.24099070834628</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4214192495081644</v>
+        <v>0.4249356230263151</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.9229580296205662</v>
+        <v>-12.88473165907399</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6690</v>
+        <v>6756</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>安碁資訊</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>260.2269505401395</v>
+        <v>262.9967487218146</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>165</v>
+        <v>94</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.66805934429847</v>
+        <v>45.33000307534098</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>19.21763596547389</v>
+        <v>18.79812087559853</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.511288706889909</v>
+        <v>0.4214192495081644</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.018831033617948</v>
+        <v>-0.9229580296205662</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6486</v>
+        <v>6690</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>互動</t>
+          <t>安碁資訊</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>257.4468650198734</v>
+        <v>260.2269505401395</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>76.8</v>
+        <v>165</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>34.0123698949042</v>
+        <v>46.66805934429847</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>22.55702216878353</v>
+        <v>19.21763596547389</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.1458818330531497</v>
+        <v>0.511288706889909</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.719417973470025</v>
+        <v>-0.018831033617948</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6674</v>
+        <v>6486</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>互動</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>247.8918210366904</v>
+        <v>257.4468650198734</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>16.3</v>
+        <v>76.8</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.09423286478997</v>
+        <v>34.0123698949042</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>19.71578864336199</v>
+        <v>22.55702216878353</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.4142206997942651</v>
+        <v>0.1458818330531497</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.0447280605718727</v>
+        <v>-0.719417973470025</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6835</v>
+        <v>6674</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>246.6147635884525</v>
+        <v>247.8918210366904</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>32.05</v>
+        <v>16.3</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>29.22304665598682</v>
+        <v>42.09423286478997</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>37.8422528040501</v>
+        <v>19.71578864336199</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.5487842990186886</v>
+        <v>0.4142206997942651</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.2247812817796377</v>
+        <v>-0.0447280605718727</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6552</v>
+        <v>6835</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>圓裕</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>246.5030053776588</v>
+        <v>246.6147635884525</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>25.45</v>
+        <v>32.05</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>34.06193643995168</v>
+        <v>29.22304665598682</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.8527996800003</v>
+        <v>37.8422528040501</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6465696005239088</v>
+        <v>0.5487842990186886</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.4777348133001298</v>
+        <v>-0.2247812817796377</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6546</v>
+        <v>6552</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>210.8314578246463</v>
+        <v>246.5030053776588</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>60.2</v>
+        <v>25.45</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,16 +6647,16 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>33.40537912008796</v>
+        <v>34.06193643995168</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>23.481648436826</v>
+        <v>16.8527996800003</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4497836352149343</v>
+        <v>0.6465696005239088</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.9479966048836376</v>
+        <v>-0.4777348133001298</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6591</v>
+        <v>6546</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>206.4489012878619</v>
+        <v>210.8314578246463</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>44.1</v>
+        <v>60.2</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>24.67207001447457</v>
+        <v>33.40537912008796</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>38.98824280088215</v>
+        <v>23.481648436826</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.5197305942258954</v>
+        <v>0.4497836352149343</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.8142380579858601</v>
+        <v>-0.9479966048836376</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6728,21 +6728,21 @@
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6838</v>
+        <v>6591</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>204.5637071380199</v>
+        <v>206.4489012878619</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>23.45</v>
+        <v>44.1</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>41.7399934561075</v>
+        <v>24.67207001447457</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>10.89058619642232</v>
+        <v>38.98824280088215</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.4960735106752635</v>
+        <v>0.5197305942258954</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0257172220109971</v>
+        <v>-0.8142380579858601</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6708</v>
+        <v>6838</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>201.8860641740236</v>
+        <v>204.5637071380199</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>38.05</v>
+        <v>23.45</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,16 +6806,16 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>42.81359504241211</v>
+        <v>41.7399934561075</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.94968348450432</v>
+        <v>10.89058619642232</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.0716187809090405</v>
+        <v>0.4960735106752635</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.219017590405012</v>
+        <v>-0.0257172220109971</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6558</v>
+        <v>6708</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>162.1525251414326</v>
+        <v>201.8860641740236</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>27.45</v>
+        <v>38.05</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>38.74031082618061</v>
+        <v>42.81359504241211</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>19.25715854698828</v>
+        <v>14.94968348450432</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.3643511127100144</v>
+        <v>0.0716187809090405</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.2508119485690615</v>
+        <v>-0.219017590405012</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6668</v>
+        <v>6558</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>155.5518532902215</v>
+        <v>162.1525251414326</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>34.15</v>
+        <v>27.45</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>33.49704709183723</v>
+        <v>38.74031082618061</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>18.91227268114985</v>
+        <v>19.25715854698828</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.3481572483782221</v>
+        <v>0.3643511127100144</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.5581484967207216</v>
+        <v>-0.2508119485690615</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6692</v>
+        <v>6668</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>143.4082445295685</v>
+        <v>155.5518532902215</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>23.85</v>
+        <v>34.15</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>41.50750762227083</v>
+        <v>33.49704709183723</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>14.36548468270474</v>
+        <v>18.91227268114985</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.766075622980061</v>
+        <v>0.3481572483782221</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.138019164096932</v>
+        <v>-0.5581484967207216</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6597</v>
+        <v>6692</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>進能服</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>114.4567076902305</v>
+        <v>143.4082445295685</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>63</v>
+        <v>23.85</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,16 +7018,16 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>49.43845693216161</v>
+        <v>41.50750762227083</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>10.00574303568831</v>
+        <v>14.36548468270474</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.1616695114489066</v>
+        <v>0.766075622980061</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.5876613289396766</v>
+        <v>-0.138019164096932</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6614</v>
+        <v>6597</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>103.672790128309</v>
+        <v>114.4567076902305</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>38.5</v>
+        <v>63</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>37.53117863650521</v>
+        <v>49.43845693216161</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.14961614914514</v>
+        <v>10.00574303568831</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.4434190217436916</v>
+        <v>0.1616695114489066</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,31 +7089,31 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.182696882199034</v>
+        <v>0.5876613289396766</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6625</v>
+        <v>6614</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>100.493407312808</v>
+        <v>103.672790128309</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>75.90000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,13 +7124,13 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>40.64762140190736</v>
+        <v>37.53117863650521</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>19.45435931709484</v>
+        <v>17.14961614914514</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.4997817865721476</v>
+        <v>0.4434190217436916</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.5062018041743038</v>
+        <v>-0.182696882199034</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7152,52 +7152,105 @@
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
+        <v>6625</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>必應</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>100.493407312808</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>40.64762140190736</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>19.45435931709484</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>0.4997817865721476</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>-0.5062018041743038</v>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
         <v>6771</v>
       </c>
-      <c r="B127" s="2" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>平和環保-創</t>
         </is>
       </c>
-      <c r="C127" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D127" s="2" t="n">
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
         <v>84.21251720866316</v>
       </c>
-      <c r="E127" s="2" t="n">
+      <c r="E128" s="2" t="n">
         <v>38.5</v>
       </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="G127" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H127" s="2" t="n">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>37.82140278697361</v>
       </c>
-      <c r="I127" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>15.42133397883871</v>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J128" s="2" t="n">
         <v>0.8861703763036319</v>
       </c>
-      <c r="K127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N127" s="2" t="n">
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
         <v>0.0139982750437389</v>
       </c>
-      <c r="O127" s="2" t="inlineStr">
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>